<commit_message>
fix: corrige nome para Clinica Inove e forca hl=pt-BR no Google Maps
</commit_message>
<xml_diff>
--- a/leads_prontos.xlsx
+++ b/leads_prontos.xlsx
@@ -465,9 +465,9 @@
   <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="99" customWidth="1" min="3" max="3"/>
+    <col width="103" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -490,85 +490,85 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Clínica Teixeira Odontologia</t>
+          <t>Clínica Inove</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>5573999990080</t>
+          <t>5573991487816</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>https://jaimilsonssdev-hue.github.io/sites-e-prospeccao/sites/clinica-teixeira-odontologia/</t>
+          <t>https://jaimilsonssdev-hue.github.io/sites-e-prospeccao/sites/clinica-inove/</t>
         </is>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Inovar Odontologia e Estética</t>
+          <t>Clínica Medic Saúde</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>557399641198</t>
+          <t>5573999950060</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>https://jaimilsonssdev-hue.github.io/sites-e-prospeccao/sites/inovar-odontologia-e-estetica/</t>
+          <t>https://jaimilsonssdev-hue.github.io/sites-e-prospeccao/sites/clinica-medic-saude/</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Biodente Odontologia</t>
+          <t>CEMED - Centro Médico Jardim Caraípe</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>5573999082467</t>
+          <t>557332914288</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>https://jaimilsonssdev-hue.github.io/sites-e-prospeccao/sites/biodente-odontologia/</t>
+          <t>https://jaimilsonssdev-hue.github.io/sites-e-prospeccao/sites/cemed-centro-medico-jardim-caraipe/</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Clínica Odontológica Sorriso</t>
+          <t>Policlínica RMed</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>557332914899</t>
+          <t>5573998608747</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>https://jaimilsonssdev-hue.github.io/sites-e-prospeccao/sites/clinica-odontologica-sorriso/</t>
+          <t>https://jaimilsonssdev-hue.github.io/sites-e-prospeccao/sites/policlinica-rmed/</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Clínica Sorridente Especializada</t>
+          <t>Clínica Prevclin - Sua Clínica Popular</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>557330131757</t>
+          <t>5573999006161</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>https://jaimilsonssdev-hue.github.io/sites-e-prospeccao/sites/clinica-sorridente-especializada/</t>
+          <t>https://jaimilsonssdev-hue.github.io/sites-e-prospeccao/sites/clinica-prevclin-sua-clinica-popular/</t>
         </is>
       </c>
     </row>

</xml_diff>